<commit_message>
test(G.8): integration tests with real Excel fixture
- Add 5 integration tests using Libro_COMPRAS_VENTAS_Ficticio.xlsx
- Regenerate fixture with cached numeric values (was formulas without
  cache -> openpyxl data_only=True returned None)
- Fix parser: remove read_only=True in openpyxl load (incompatible with
  index-based row access, gave empty rows)
- Add 'iva importacion 16%' header alias (fixture header lacks 'de')
- Test test_import_real_fixture_purchase_totals_matches_excel hardcodes
  expected totals to detect fixture mutations
- Helper _compute_expected_totals_from_fixture combines base_import_16
  into base_general (matches _build_vat_book_vals behavior)

Mutation test: changing fixture base_general row 8 col 23 from
818896.74 to 999999.99 makes the test fail with 181103.25 difference.

Tests: 0 failed, 0 error(s) of 96 tests
</commit_message>
<xml_diff>
--- a/addons/l10n_ve_compliance_manager/tests/fixtures/Libro_COMPRAS_VENTAS_Ficticio.xlsx
+++ b/addons/l10n_ve_compliance_manager/tests/fixtures/Libro_COMPRAS_VENTAS_Ficticio.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE27"/>
+  <dimension ref="B1:AE27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -828,9 +828,8 @@
       <c r="W8" s="6" t="n">
         <v>818896.74</v>
       </c>
-      <c r="X8" s="6">
-        <f>IF(Q8&gt;0, ROUND((P8-U8-V8-S8)/1.16, 2), 0)</f>
-        <v/>
+      <c r="X8" s="6" t="n">
+        <v>131023.48</v>
       </c>
       <c r="Y8" s="6">
         <f>ROUND(W8*0.16, 2)</f>
@@ -852,9 +851,8 @@
       <c r="AC8" s="6" t="n">
         <v>98267.61</v>
       </c>
-      <c r="AD8" s="6">
-        <f>IF(AA8&lt;&gt;"", ROUND(X8*0.75, 2), 0)</f>
-        <v/>
+      <c r="AD8" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="AE8" s="6" t="n">
         <v>0</v>
@@ -929,9 +927,8 @@
       <c r="W9" s="6" t="n">
         <v>258620.69</v>
       </c>
-      <c r="X9" s="6">
-        <f>IF(Q9&gt;0, ROUND((P9-U9-V9-S9)/1.16, 2), 0)</f>
-        <v/>
+      <c r="X9" s="6" t="n">
+        <v>41379.31</v>
       </c>
       <c r="Y9" s="6">
         <f>ROUND(W9*0.16, 2)</f>
@@ -953,9 +950,8 @@
       <c r="AC9" s="6" t="n">
         <v>31034.48</v>
       </c>
-      <c r="AD9" s="6">
-        <f>IF(AA9&lt;&gt;"", ROUND(X9*0.75, 2), 0)</f>
-        <v/>
+      <c r="AD9" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="AE9" s="6" t="n">
         <v>0</v>
@@ -1030,9 +1026,8 @@
       <c r="W10" s="6" t="n">
         <v>155172.41</v>
       </c>
-      <c r="X10" s="6">
-        <f>IF(Q10&gt;0, ROUND((P10-U10-V10-S10)/1.16, 2), 0)</f>
-        <v/>
+      <c r="X10" s="6" t="n">
+        <v>24827.59</v>
       </c>
       <c r="Y10" s="6">
         <f>ROUND(W10*0.16, 2)</f>
@@ -1054,9 +1049,8 @@
       <c r="AC10" s="6" t="n">
         <v>18620.69</v>
       </c>
-      <c r="AD10" s="6">
-        <f>IF(AA10&lt;&gt;"", ROUND(X10*0.75, 2), 0)</f>
-        <v/>
+      <c r="AD10" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="AE10" s="6" t="n">
         <v>0</v>
@@ -1131,9 +1125,8 @@
       <c r="W11" s="6" t="n">
         <v>189655.17</v>
       </c>
-      <c r="X11" s="6">
-        <f>IF(Q11&gt;0, ROUND((P11-U11-V11-S11)/1.16, 2), 0)</f>
-        <v/>
+      <c r="X11" s="6" t="n">
+        <v>30344.83</v>
       </c>
       <c r="Y11" s="6">
         <f>ROUND(W11*0.16, 2)</f>
@@ -1155,9 +1148,8 @@
       <c r="AC11" s="6" t="n">
         <v>22758.62</v>
       </c>
-      <c r="AD11" s="6">
-        <f>IF(AA11&lt;&gt;"", ROUND(X11*0.75, 2), 0)</f>
-        <v/>
+      <c r="AD11" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="AE11" s="6" t="n">
         <v>0</v>
@@ -1232,9 +1224,8 @@
       <c r="W12" s="6" t="n">
         <v>81896.55</v>
       </c>
-      <c r="X12" s="6">
-        <f>IF(Q12&gt;0, ROUND((P12-U12-V12-S12)/1.16, 2), 0)</f>
-        <v/>
+      <c r="X12" s="6" t="n">
+        <v>13103.45</v>
       </c>
       <c r="Y12" s="6">
         <f>ROUND(W12*0.16, 2)</f>
@@ -1256,9 +1247,8 @@
       <c r="AC12" s="6" t="n">
         <v>9827.59</v>
       </c>
-      <c r="AD12" s="6">
-        <f>IF(AA12&lt;&gt;"", ROUND(X12*0.75, 2), 0)</f>
-        <v/>
+      <c r="AD12" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="AE12" s="6" t="n">
         <v>0</v>
@@ -1345,9 +1335,8 @@
       <c r="W13" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="X13" s="6">
-        <f>IF(Q13&gt;0, ROUND((P13-U13-V13-S13)/1.16, 2), 0)</f>
-        <v/>
+      <c r="X13" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="Y13" s="6">
         <f>ROUND(W13*0.16, 2)</f>
@@ -1361,9 +1350,8 @@
       <c r="AC13" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AD13" s="6">
-        <f>IF(AA13&lt;&gt;"", ROUND(X13*0.75, 2), 0)</f>
-        <v/>
+      <c r="AD13" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="AE13" s="6" t="n">
         <v>64000</v>
@@ -1438,9 +1426,8 @@
       <c r="W14" s="6" t="n">
         <v>125000</v>
       </c>
-      <c r="X14" s="6">
-        <f>IF(Q14&gt;0, ROUND((P14-U14-V14-S14)/1.16, 2), 0)</f>
-        <v/>
+      <c r="X14" s="6" t="n">
+        <v>20000</v>
       </c>
       <c r="Y14" s="6">
         <f>ROUND(W14*0.16, 2)</f>
@@ -1462,9 +1449,8 @@
       <c r="AC14" s="6" t="n">
         <v>15000</v>
       </c>
-      <c r="AD14" s="6">
-        <f>IF(AA14&lt;&gt;"", ROUND(X14*0.75, 2), 0)</f>
-        <v/>
+      <c r="AD14" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="AE14" s="6" t="n">
         <v>0</v>
@@ -1539,9 +1525,8 @@
       <c r="W15" s="6" t="n">
         <v>362068.97</v>
       </c>
-      <c r="X15" s="6">
-        <f>IF(Q15&gt;0, ROUND((P15-U15-V15-S15)/1.16, 2), 0)</f>
-        <v/>
+      <c r="X15" s="6" t="n">
+        <v>57931.04</v>
       </c>
       <c r="Y15" s="6">
         <f>ROUND(W15*0.16, 2)</f>
@@ -1561,11 +1546,10 @@
         </is>
       </c>
       <c r="AC15" s="6" t="n">
-        <v>43448.27</v>
-      </c>
-      <c r="AD15" s="6">
-        <f>IF(AA15&lt;&gt;"", ROUND(X15*0.75, 2), 0)</f>
-        <v/>
+        <v>43448.28</v>
+      </c>
+      <c r="AD15" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="AE15" s="6" t="n">
         <v>0</v>
@@ -1640,9 +1624,8 @@
       <c r="W16" s="6" t="n">
         <v>86206.89999999999</v>
       </c>
-      <c r="X16" s="6">
-        <f>IF(Q16&gt;0, ROUND((P16-U16-V16-S16)/1.16, 2), 0)</f>
-        <v/>
+      <c r="X16" s="6" t="n">
+        <v>13793.1</v>
       </c>
       <c r="Y16" s="6">
         <f>ROUND(W16*0.16, 2)</f>
@@ -1664,9 +1647,8 @@
       <c r="AC16" s="6" t="n">
         <v>10344.83</v>
       </c>
-      <c r="AD16" s="6">
-        <f>IF(AA16&lt;&gt;"", ROUND(X16*0.75, 2), 0)</f>
-        <v/>
+      <c r="AD16" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="AE16" s="6" t="n">
         <v>0</v>
@@ -1741,9 +1723,8 @@
       <c r="W17" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="X17" s="6">
-        <f>IF(Q17&gt;0, ROUND((P17-U17-V17-S17)/1.16, 2), 0)</f>
-        <v/>
+      <c r="X17" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="Y17" s="6">
         <f>ROUND(W17*0.16, 2)</f>
@@ -1757,9 +1738,8 @@
       <c r="AC17" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AD17" s="6">
-        <f>IF(AA17&lt;&gt;"", ROUND(X17*0.75, 2), 0)</f>
-        <v/>
+      <c r="AD17" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="AE17" s="6" t="n">
         <v>0</v>
@@ -1824,8 +1804,6 @@
         <v/>
       </c>
     </row>
-    <row r="19"/>
-    <row r="20"/>
     <row r="21">
       <c r="D21" s="2" t="inlineStr">
         <is>
@@ -1969,7 +1947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB34"/>
+  <dimension ref="B5:AB34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2002,10 +1980,6 @@
     <col width="25" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -2061,7 +2035,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="B11" s="3" t="inlineStr">
         <is>
@@ -2258,9 +2231,8 @@
       <c r="S12" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="T12" s="6">
-        <f>ROUND(R12*0.16, 2)</f>
-        <v/>
+      <c r="T12" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="U12" s="6" t="n">
         <v>0</v>
@@ -2271,9 +2243,8 @@
       <c r="W12" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="X12" s="6">
-        <f>ROUND(V12*0.16, 2)</f>
-        <v/>
+      <c r="X12" s="6" t="n">
+        <v>12349.34</v>
       </c>
       <c r="Y12" s="4" t="inlineStr">
         <is>
@@ -2351,9 +2322,8 @@
       <c r="S13" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="T13" s="6">
-        <f>ROUND(R13*0.16, 2)</f>
-        <v/>
+      <c r="T13" s="6" t="n">
+        <v>16465.96</v>
       </c>
       <c r="U13" s="6" t="n">
         <v>0</v>
@@ -2364,9 +2334,8 @@
       <c r="W13" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="X13" s="6">
-        <f>ROUND(V13*0.16, 2)</f>
-        <v/>
+      <c r="X13" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="Y13" s="4" t="inlineStr"/>
       <c r="Z13" s="4" t="inlineStr"/>
@@ -2436,9 +2405,8 @@
       <c r="S14" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="T14" s="6">
-        <f>ROUND(R14*0.16, 2)</f>
-        <v/>
+      <c r="T14" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="U14" s="6" t="n">
         <v>0</v>
@@ -2449,9 +2417,8 @@
       <c r="W14" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="X14" s="6">
-        <f>ROUND(V14*0.16, 2)</f>
-        <v/>
+      <c r="X14" s="6" t="n">
+        <v>18302.16</v>
       </c>
       <c r="Y14" s="4" t="inlineStr">
         <is>
@@ -2464,7 +2431,7 @@
         </is>
       </c>
       <c r="AA14" s="6" t="n">
-        <v>13726.63</v>
+        <v>13726.62</v>
       </c>
       <c r="AB14" s="6" t="n">
         <v>4575.54</v>
@@ -2529,9 +2496,8 @@
       <c r="S15" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="T15" s="6">
-        <f>ROUND(R15*0.16, 2)</f>
-        <v/>
+      <c r="T15" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="U15" s="6" t="n">
         <v>0</v>
@@ -2542,9 +2508,8 @@
       <c r="W15" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="X15" s="6">
-        <f>ROUND(V15*0.16, 2)</f>
-        <v/>
+      <c r="X15" s="6" t="n">
+        <v>4194.68</v>
       </c>
       <c r="Y15" s="4" t="inlineStr">
         <is>
@@ -2557,7 +2522,7 @@
         </is>
       </c>
       <c r="AA15" s="6" t="n">
-        <v>3146</v>
+        <v>3146.01</v>
       </c>
       <c r="AB15" s="6" t="n">
         <v>1048.67</v>
@@ -2622,9 +2587,8 @@
       <c r="S16" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="T16" s="6">
-        <f>ROUND(R16*0.16, 2)</f>
-        <v/>
+      <c r="T16" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="U16" s="6" t="n">
         <v>0</v>
@@ -2635,9 +2599,8 @@
       <c r="W16" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="X16" s="6">
-        <f>ROUND(V16*0.16, 2)</f>
-        <v/>
+      <c r="X16" s="6" t="n">
+        <v>3597.58</v>
       </c>
       <c r="Y16" s="4" t="inlineStr">
         <is>
@@ -2650,7 +2613,7 @@
         </is>
       </c>
       <c r="AA16" s="6" t="n">
-        <v>2698.19</v>
+        <v>2698.18</v>
       </c>
       <c r="AB16" s="6" t="n">
         <v>899.39</v>
@@ -2711,9 +2674,8 @@
       <c r="S17" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="T17" s="6">
-        <f>ROUND(R17*0.16, 2)</f>
-        <v/>
+      <c r="T17" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="U17" s="6" t="n">
         <v>0</v>
@@ -2724,9 +2686,8 @@
       <c r="W17" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="X17" s="6">
-        <f>ROUND(V17*0.16, 2)</f>
-        <v/>
+      <c r="X17" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="Y17" s="4" t="inlineStr"/>
       <c r="Z17" s="4" t="inlineStr"/>
@@ -2796,9 +2757,8 @@
       <c r="S18" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="T18" s="6">
-        <f>ROUND(R18*0.16, 2)</f>
-        <v/>
+      <c r="T18" s="6" t="n">
+        <v>18957.39</v>
       </c>
       <c r="U18" s="6" t="n">
         <v>0</v>
@@ -2809,9 +2769,8 @@
       <c r="W18" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="X18" s="6">
-        <f>ROUND(V18*0.16, 2)</f>
-        <v/>
+      <c r="X18" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="Y18" s="4" t="inlineStr"/>
       <c r="Z18" s="4" t="inlineStr"/>
@@ -2881,9 +2840,8 @@
       <c r="S19" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="T19" s="6">
-        <f>ROUND(R19*0.16, 2)</f>
-        <v/>
+      <c r="T19" s="6" t="n">
+        <v>18831.85</v>
       </c>
       <c r="U19" s="6" t="n">
         <v>0</v>
@@ -2894,9 +2852,8 @@
       <c r="W19" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="X19" s="6">
-        <f>ROUND(V19*0.16, 2)</f>
-        <v/>
+      <c r="X19" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="Y19" s="4" t="inlineStr"/>
       <c r="Z19" s="4" t="inlineStr"/>
@@ -2966,9 +2923,8 @@
       <c r="S20" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="T20" s="6">
-        <f>ROUND(R20*0.16, 2)</f>
-        <v/>
+      <c r="T20" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="U20" s="6" t="n">
         <v>0</v>
@@ -2979,9 +2935,8 @@
       <c r="W20" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="X20" s="6">
-        <f>ROUND(V20*0.16, 2)</f>
-        <v/>
+      <c r="X20" s="6" t="n">
+        <v>1271.98</v>
       </c>
       <c r="Y20" s="4" t="inlineStr">
         <is>
@@ -3059,9 +3014,8 @@
       <c r="S21" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="T21" s="6">
-        <f>ROUND(R21*0.16, 2)</f>
-        <v/>
+      <c r="T21" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="U21" s="6" t="n">
         <v>12500</v>
@@ -3072,9 +3026,8 @@
       <c r="W21" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="X21" s="6">
-        <f>ROUND(V21*0.16, 2)</f>
-        <v/>
+      <c r="X21" s="6" t="n">
+        <v>11862.07</v>
       </c>
       <c r="Y21" s="4" t="inlineStr">
         <is>
@@ -3140,8 +3093,6 @@
         <v/>
       </c>
     </row>
-    <row r="23"/>
-    <row r="24"/>
     <row r="25">
       <c r="D25" s="2" t="inlineStr">
         <is>
@@ -3428,7 +3379,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
         <is>

</xml_diff>